<commit_message>
Enhance watchlist feature to support Excel input files
- parser.py: add read_excel_and_parse() to read Symbol/Name/Exchange
  from .xlsx input files (supports Companies and Stocks sheet names,
  case-insensitive column matching)
- watchlist_to_excel.py: dispatch on file extension (.txt vs .xlsx);
  Excel input removes processed rows from the input file after writing
  to A2ZStocks.xlsx; refactored shared logic into _save_output()
- modules/__init__.py: export read_excel_and_parse
- outputs/A2ZStocks.xlsx: updated with Total row in Summary sheet

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/A2ZStocks.xlsx
+++ b/outputs/A2ZStocks.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D608"/>
+  <dimension ref="A1:D610"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8106,17 +8106,17 @@
     <row r="353">
       <c r="A353" s="3" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>NEWX</t>
         </is>
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>Netflix</t>
+          <t>New Company X</t>
         </is>
       </c>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D353" s="3" t="inlineStr">
@@ -8128,17 +8128,17 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>NIO</t>
+          <t>NEWY</t>
         </is>
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>NIO</t>
+          <t>New Company Y</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -8150,13 +8150,17 @@
     <row r="355">
       <c r="A355" s="3" t="inlineStr">
         <is>
-          <t>NKE</t>
-        </is>
-      </c>
-      <c r="B355" s="3" t="n"/>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="B355" s="3" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D355" s="3" t="inlineStr">
@@ -8168,12 +8172,12 @@
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>NNVC</t>
+          <t>NIO</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>NanoViricides</t>
+          <t>NIO</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
@@ -8190,14 +8194,10 @@
     <row r="357">
       <c r="A357" s="3" t="inlineStr">
         <is>
-          <t>NOC</t>
-        </is>
-      </c>
-      <c r="B357" s="3" t="inlineStr">
-        <is>
-          <t>Northrop Grumman</t>
-        </is>
-      </c>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="B357" s="3" t="n"/>
       <c r="C357" s="3" t="inlineStr">
         <is>
           <t>NYSE</t>
@@ -8212,12 +8212,12 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>NNVC</t>
         </is>
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>Nokia Corporation</t>
+          <t>NanoViricides</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
@@ -8234,10 +8234,14 @@
     <row r="359">
       <c r="A359" s="3" t="inlineStr">
         <is>
-          <t>NOW</t>
-        </is>
-      </c>
-      <c r="B359" s="3" t="n"/>
+          <t>NOC</t>
+        </is>
+      </c>
+      <c r="B359" s="3" t="inlineStr">
+        <is>
+          <t>Northrop Grumman</t>
+        </is>
+      </c>
       <c r="C359" s="3" t="inlineStr">
         <is>
           <t>NYSE</t>
@@ -8252,17 +8256,17 @@
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>NerdWallet</t>
+          <t>Nokia Corporation</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -8274,14 +8278,10 @@
     <row r="361">
       <c r="A361" s="3" t="inlineStr">
         <is>
-          <t>NRGV</t>
-        </is>
-      </c>
-      <c r="B361" s="3" t="inlineStr">
-        <is>
-          <t>Energy Vault</t>
-        </is>
-      </c>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B361" s="3" t="n"/>
       <c r="C361" s="3" t="inlineStr">
         <is>
           <t>NYSE</t>
@@ -8296,12 +8296,12 @@
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>NRDS</t>
         </is>
       </c>
       <c r="B362" s="2" t="inlineStr">
         <is>
-          <t>NetApp</t>
+          <t>NerdWallet</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
@@ -8318,17 +8318,17 @@
     <row r="363">
       <c r="A363" s="3" t="inlineStr">
         <is>
-          <t>NTRS</t>
+          <t>NRGV</t>
         </is>
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>Northern Trust</t>
+          <t>Energy Vault</t>
         </is>
       </c>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D363" s="3" t="inlineStr">
@@ -8340,17 +8340,17 @@
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>NUKZ</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="B364" s="2" t="inlineStr">
         <is>
-          <t>Range Nuclear Renaissance Index ETF</t>
+          <t>NetApp</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -8362,12 +8362,12 @@
     <row r="365">
       <c r="A365" s="3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>NTRS</t>
         </is>
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>NVIDIA .</t>
+          <t>Northern Trust</t>
         </is>
       </c>
       <c r="C365" s="3" t="inlineStr">
@@ -8384,17 +8384,17 @@
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>NVDL</t>
+          <t>NUKZ</t>
         </is>
       </c>
       <c r="B366" s="2" t="inlineStr">
         <is>
-          <t>GraniteShares 2x Long NVDA Daily ETF</t>
+          <t>Range Nuclear Renaissance Index ETF</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
@@ -8406,12 +8406,12 @@
     <row r="367">
       <c r="A367" s="3" t="inlineStr">
         <is>
-          <t>NVMI</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>Nova Ltd.</t>
+          <t>NVIDIA .</t>
         </is>
       </c>
       <c r="C367" s="3" t="inlineStr">
@@ -8428,13 +8428,17 @@
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>NVO</t>
-        </is>
-      </c>
-      <c r="B368" s="2" t="n"/>
+          <t>NVDL</t>
+        </is>
+      </c>
+      <c r="B368" s="2" t="inlineStr">
+        <is>
+          <t>GraniteShares 2x Long NVDA Daily ETF</t>
+        </is>
+      </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
@@ -8446,17 +8450,17 @@
     <row r="369">
       <c r="A369" s="3" t="inlineStr">
         <is>
-          <t>NVS</t>
+          <t>NVMI</t>
         </is>
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>Nova Ltd.</t>
         </is>
       </c>
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D369" s="3" t="inlineStr">
@@ -8468,17 +8472,13 @@
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>NXT</t>
-        </is>
-      </c>
-      <c r="B370" s="2" t="inlineStr">
-        <is>
-          <t>Nextpower</t>
-        </is>
-      </c>
+          <t>NVO</t>
+        </is>
+      </c>
+      <c r="B370" s="2" t="n"/>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
@@ -8490,12 +8490,12 @@
     <row r="371">
       <c r="A371" s="3" t="inlineStr">
         <is>
-          <t>NYT</t>
+          <t>NVS</t>
         </is>
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>The New York Times</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="C371" s="3" t="inlineStr">
@@ -8512,17 +8512,17 @@
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B372" s="2" t="inlineStr">
         <is>
-          <t>Realty Income</t>
+          <t>Nextpower</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
@@ -8534,12 +8534,12 @@
     <row r="373">
       <c r="A373" s="3" t="inlineStr">
         <is>
-          <t>OHI</t>
+          <t>NYT</t>
         </is>
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>Omega Healthcare Investors</t>
+          <t>The New York Times</t>
         </is>
       </c>
       <c r="C373" s="3" t="inlineStr">
@@ -8556,12 +8556,12 @@
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>OKLO</t>
+          <t>O</t>
         </is>
       </c>
       <c r="B374" s="2" t="inlineStr">
         <is>
-          <t>Oklo</t>
+          <t>Realty Income</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
@@ -8578,17 +8578,17 @@
     <row r="375">
       <c r="A375" s="3" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>OHI</t>
         </is>
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>Okta</t>
+          <t>Omega Healthcare Investors</t>
         </is>
       </c>
       <c r="C375" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D375" s="3" t="inlineStr">
@@ -8600,13 +8600,17 @@
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>OLLI</t>
-        </is>
-      </c>
-      <c r="B376" s="2" t="n"/>
+          <t>OKLO</t>
+        </is>
+      </c>
+      <c r="B376" s="2" t="inlineStr">
+        <is>
+          <t>Oklo</t>
+        </is>
+      </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D376" s="2" t="inlineStr">
@@ -8618,12 +8622,12 @@
     <row r="377">
       <c r="A377" s="3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OKTA</t>
         </is>
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>Okta</t>
         </is>
       </c>
       <c r="C377" s="3" t="inlineStr">
@@ -8640,7 +8644,7 @@
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>ONDS</t>
+          <t>OLLI</t>
         </is>
       </c>
       <c r="B378" s="2" t="n"/>
@@ -8658,17 +8662,17 @@
     <row r="379">
       <c r="A379" s="3" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>On Holdings</t>
+          <t>onsemi</t>
         </is>
       </c>
       <c r="C379" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D379" s="3" t="inlineStr">
@@ -8680,7 +8684,7 @@
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>ONDS</t>
         </is>
       </c>
       <c r="B380" s="2" t="n"/>
@@ -8698,12 +8702,12 @@
     <row r="381">
       <c r="A381" s="3" t="inlineStr">
         <is>
-          <t>ORA</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>Ormat Technologies</t>
+          <t>On Holdings</t>
         </is>
       </c>
       <c r="C381" s="3" t="inlineStr">
@@ -8720,17 +8724,13 @@
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>ORCL</t>
-        </is>
-      </c>
-      <c r="B382" s="2" t="inlineStr">
-        <is>
-          <t>Oracle Corporation</t>
-        </is>
-      </c>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="B382" s="2" t="n"/>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
@@ -8742,13 +8742,17 @@
     <row r="383">
       <c r="A383" s="3" t="inlineStr">
         <is>
-          <t>ORLY</t>
-        </is>
-      </c>
-      <c r="B383" s="3" t="n"/>
+          <t>ORA</t>
+        </is>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>Ormat Technologies</t>
+        </is>
+      </c>
       <c r="C383" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D383" s="3" t="inlineStr">
@@ -8760,12 +8764,12 @@
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>OSCR</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B384" s="2" t="inlineStr">
         <is>
-          <t>Oscar Health</t>
+          <t>Oracle Corporation</t>
         </is>
       </c>
       <c r="C384" s="2" t="inlineStr">
@@ -8782,17 +8786,13 @@
     <row r="385">
       <c r="A385" s="3" t="inlineStr">
         <is>
-          <t>OWL</t>
-        </is>
-      </c>
-      <c r="B385" s="3" t="inlineStr">
-        <is>
-          <t>Blue Owl Capital</t>
-        </is>
-      </c>
+          <t>ORLY</t>
+        </is>
+      </c>
+      <c r="B385" s="3" t="n"/>
       <c r="C385" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D385" s="3" t="inlineStr">
@@ -8804,12 +8804,12 @@
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>OXY</t>
+          <t>OSCR</t>
         </is>
       </c>
       <c r="B386" s="2" t="inlineStr">
         <is>
-          <t>Occidental Petroleum</t>
+          <t>Oscar Health</t>
         </is>
       </c>
       <c r="C386" s="2" t="inlineStr">
@@ -8826,17 +8826,17 @@
     <row r="387">
       <c r="A387" s="3" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>OWL</t>
         </is>
       </c>
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>Palo Alto Networks</t>
+          <t>Blue Owl Capital</t>
         </is>
       </c>
       <c r="C387" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D387" s="3" t="inlineStr">
@@ -8848,12 +8848,12 @@
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>OXY</t>
         </is>
       </c>
       <c r="B388" s="2" t="inlineStr">
         <is>
-          <t>UiPath</t>
+          <t>Occidental Petroleum</t>
         </is>
       </c>
       <c r="C388" s="2" t="inlineStr">
@@ -8870,17 +8870,17 @@
     <row r="389">
       <c r="A389" s="3" t="inlineStr">
         <is>
-          <t>PAYC</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>Paycom Software</t>
+          <t>Palo Alto Networks</t>
         </is>
       </c>
       <c r="C389" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D389" s="3" t="inlineStr">
@@ -8892,17 +8892,17 @@
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>PAYP</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B390" s="2" t="inlineStr">
         <is>
-          <t>PayPay Corporation</t>
+          <t>UiPath</t>
         </is>
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D390" s="2" t="inlineStr">
@@ -8914,12 +8914,12 @@
     <row r="391">
       <c r="A391" s="3" t="inlineStr">
         <is>
-          <t>PBF</t>
+          <t>PAYC</t>
         </is>
       </c>
       <c r="B391" s="3" t="inlineStr">
         <is>
-          <t>PBF Energy</t>
+          <t>Paycom Software</t>
         </is>
       </c>
       <c r="C391" s="3" t="inlineStr">
@@ -8936,17 +8936,17 @@
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>PBT</t>
+          <t>PAYP</t>
         </is>
       </c>
       <c r="B392" s="2" t="inlineStr">
         <is>
-          <t>Permian Basin Royalty Trust</t>
+          <t>PayPay Corporation</t>
         </is>
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -8958,17 +8958,17 @@
     <row r="393">
       <c r="A393" s="3" t="inlineStr">
         <is>
-          <t>PDD</t>
+          <t>PBF</t>
         </is>
       </c>
       <c r="B393" s="3" t="inlineStr">
         <is>
-          <t>PDD</t>
+          <t>PBF Energy</t>
         </is>
       </c>
       <c r="C393" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D393" s="3" t="inlineStr">
@@ -8980,17 +8980,17 @@
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>PDYN</t>
+          <t>PBT</t>
         </is>
       </c>
       <c r="B394" s="2" t="inlineStr">
         <is>
-          <t>Palladyne AI</t>
+          <t>Permian Basin Royalty Trust</t>
         </is>
       </c>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D394" s="2" t="inlineStr">
@@ -9002,17 +9002,17 @@
     <row r="395">
       <c r="A395" s="3" t="inlineStr">
         <is>
-          <t>PEJ</t>
+          <t>PDD</t>
         </is>
       </c>
       <c r="B395" s="3" t="inlineStr">
         <is>
-          <t>Invesco Leisure and Entertainment ETF</t>
+          <t>PDD</t>
         </is>
       </c>
       <c r="C395" s="3" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D395" s="3" t="inlineStr">
@@ -9024,17 +9024,17 @@
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>PEN</t>
+          <t>PDYN</t>
         </is>
       </c>
       <c r="B396" s="2" t="inlineStr">
         <is>
-          <t>Penumbra</t>
+          <t>Palladyne AI</t>
         </is>
       </c>
       <c r="C396" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D396" s="2" t="inlineStr">
@@ -9046,17 +9046,17 @@
     <row r="397">
       <c r="A397" s="3" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>PEJ</t>
         </is>
       </c>
       <c r="B397" s="3" t="inlineStr">
         <is>
-          <t>Penguin Solutions</t>
+          <t>Invesco Leisure and Entertainment ETF</t>
         </is>
       </c>
       <c r="C397" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D397" s="3" t="inlineStr">
@@ -9068,17 +9068,17 @@
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>PEN</t>
         </is>
       </c>
       <c r="B398" s="2" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>Penumbra</t>
         </is>
       </c>
       <c r="C398" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D398" s="2" t="inlineStr">
@@ -9090,17 +9090,17 @@
     <row r="399">
       <c r="A399" s="3" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="B399" s="3" t="inlineStr">
         <is>
-          <t>Pfizer</t>
+          <t>Penguin Solutions</t>
         </is>
       </c>
       <c r="C399" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D399" s="3" t="inlineStr">
@@ -9112,17 +9112,17 @@
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B400" s="2" t="inlineStr">
         <is>
-          <t>Gamble</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="C400" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D400" s="2" t="inlineStr">
@@ -9134,12 +9134,12 @@
     <row r="401">
       <c r="A401" s="3" t="inlineStr">
         <is>
-          <t>PGR</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="B401" s="3" t="inlineStr">
         <is>
-          <t>Progressive</t>
+          <t>Pfizer</t>
         </is>
       </c>
       <c r="C401" s="3" t="inlineStr">
@@ -9156,17 +9156,17 @@
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>PGY</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B402" s="2" t="inlineStr">
         <is>
-          <t>Pagaya Technologies</t>
+          <t>Gamble</t>
         </is>
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -9178,12 +9178,12 @@
     <row r="403">
       <c r="A403" s="3" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PGR</t>
         </is>
       </c>
       <c r="B403" s="3" t="inlineStr">
         <is>
-          <t>Planet Labs PBC</t>
+          <t>Progressive</t>
         </is>
       </c>
       <c r="C403" s="3" t="inlineStr">
@@ -9200,12 +9200,12 @@
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>PGY</t>
         </is>
       </c>
       <c r="B404" s="2" t="inlineStr">
         <is>
-          <t>Photronics</t>
+          <t>Pagaya Technologies</t>
         </is>
       </c>
       <c r="C404" s="2" t="inlineStr">
@@ -9222,17 +9222,17 @@
     <row r="405">
       <c r="A405" s="3" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="B405" s="3" t="inlineStr">
         <is>
-          <t>Buster's</t>
+          <t>Planet Labs PBC</t>
         </is>
       </c>
       <c r="C405" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D405" s="3" t="inlineStr">
@@ -9244,13 +9244,17 @@
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>PLD</t>
-        </is>
-      </c>
-      <c r="B406" s="2" t="n"/>
+          <t>PLAB</t>
+        </is>
+      </c>
+      <c r="B406" s="2" t="inlineStr">
+        <is>
+          <t>Photronics</t>
+        </is>
+      </c>
       <c r="C406" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D406" s="2" t="inlineStr">
@@ -9262,12 +9266,12 @@
     <row r="407">
       <c r="A407" s="3" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>PLAY</t>
         </is>
       </c>
       <c r="B407" s="3" t="inlineStr">
         <is>
-          <t>Palantir</t>
+          <t>Buster's</t>
         </is>
       </c>
       <c r="C407" s="3" t="inlineStr">
@@ -9284,17 +9288,13 @@
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>PMAX</t>
-        </is>
-      </c>
-      <c r="B408" s="2" t="inlineStr">
-        <is>
-          <t>Powell Max Limited</t>
-        </is>
-      </c>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="B408" s="2" t="n"/>
       <c r="C408" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D408" s="2" t="inlineStr">
@@ -9306,17 +9306,17 @@
     <row r="409">
       <c r="A409" s="3" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B409" s="3" t="inlineStr">
         <is>
-          <t>PNC Financial Services</t>
+          <t>Palantir</t>
         </is>
       </c>
       <c r="C409" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D409" s="3" t="inlineStr">
@@ -9328,12 +9328,12 @@
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>PPSI</t>
+          <t>PMAX</t>
         </is>
       </c>
       <c r="B410" s="2" t="inlineStr">
         <is>
-          <t>Pioneer Power</t>
+          <t>Powell Max Limited</t>
         </is>
       </c>
       <c r="C410" s="2" t="inlineStr">
@@ -9350,17 +9350,17 @@
     <row r="411">
       <c r="A411" s="3" t="inlineStr">
         <is>
-          <t>PPTA</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B411" s="3" t="inlineStr">
         <is>
-          <t>Perpetua Resources</t>
+          <t>PNC Financial Services</t>
         </is>
       </c>
       <c r="C411" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D411" s="3" t="inlineStr">
@@ -9372,17 +9372,17 @@
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>PRLB</t>
+          <t>PPSI</t>
         </is>
       </c>
       <c r="B412" s="2" t="inlineStr">
         <is>
-          <t>Proto Labs</t>
+          <t>Pioneer Power</t>
         </is>
       </c>
       <c r="C412" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D412" s="2" t="inlineStr">
@@ -9394,17 +9394,17 @@
     <row r="413">
       <c r="A413" s="3" t="inlineStr">
         <is>
-          <t>PSIL</t>
+          <t>PPTA</t>
         </is>
       </c>
       <c r="B413" s="3" t="inlineStr">
         <is>
-          <t>AdvisorShares Psychedelics ETF</t>
+          <t>Perpetua Resources</t>
         </is>
       </c>
       <c r="C413" s="3" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D413" s="3" t="inlineStr">
@@ -9416,17 +9416,17 @@
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>PSKY</t>
+          <t>PRLB</t>
         </is>
       </c>
       <c r="B414" s="2" t="inlineStr">
         <is>
-          <t>Paramount Skydance</t>
+          <t>Proto Labs</t>
         </is>
       </c>
       <c r="C414" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D414" s="2" t="inlineStr">
@@ -9438,17 +9438,17 @@
     <row r="415">
       <c r="A415" s="3" t="inlineStr">
         <is>
-          <t>PSMT</t>
+          <t>PSIL</t>
         </is>
       </c>
       <c r="B415" s="3" t="inlineStr">
         <is>
-          <t>PriceSmart</t>
+          <t>AdvisorShares Psychedelics ETF</t>
         </is>
       </c>
       <c r="C415" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D415" s="3" t="inlineStr">
@@ -9460,17 +9460,17 @@
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>PSTG</t>
+          <t>PSKY</t>
         </is>
       </c>
       <c r="B416" s="2" t="inlineStr">
         <is>
-          <t>Everpure</t>
+          <t>Paramount Skydance</t>
         </is>
       </c>
       <c r="C416" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D416" s="2" t="inlineStr">
@@ -9482,17 +9482,17 @@
     <row r="417">
       <c r="A417" s="3" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>PSMT</t>
         </is>
       </c>
       <c r="B417" s="3" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>PriceSmart</t>
         </is>
       </c>
       <c r="C417" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D417" s="3" t="inlineStr">
@@ -9504,17 +9504,17 @@
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>PTON</t>
+          <t>PSTG</t>
         </is>
       </c>
       <c r="B418" s="2" t="inlineStr">
         <is>
-          <t>Peloton Interactive</t>
+          <t>Everpure</t>
         </is>
       </c>
       <c r="C418" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D418" s="2" t="inlineStr">
@@ -9526,12 +9526,12 @@
     <row r="419">
       <c r="A419" s="3" t="inlineStr">
         <is>
-          <t>PVH</t>
+          <t>PSX</t>
         </is>
       </c>
       <c r="B419" s="3" t="inlineStr">
         <is>
-          <t>PVH .'s</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="C419" s="3" t="inlineStr">
@@ -9548,17 +9548,17 @@
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>PYLD</t>
+          <t>PTON</t>
         </is>
       </c>
       <c r="B420" s="2" t="inlineStr">
         <is>
-          <t>PIMCO Multisector Bond Active ETF</t>
+          <t>Peloton Interactive</t>
         </is>
       </c>
       <c r="C420" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D420" s="2" t="inlineStr">
@@ -9570,17 +9570,17 @@
     <row r="421">
       <c r="A421" s="3" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>PVH</t>
         </is>
       </c>
       <c r="B421" s="3" t="inlineStr">
         <is>
-          <t>PayPal</t>
+          <t>PVH .'s</t>
         </is>
       </c>
       <c r="C421" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D421" s="3" t="inlineStr">
@@ -9592,17 +9592,17 @@
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>PYLD</t>
         </is>
       </c>
       <c r="B422" s="2" t="inlineStr">
         <is>
-          <t>Qnity Electronics</t>
+          <t>PIMCO Multisector Bond Active ETF</t>
         </is>
       </c>
       <c r="C422" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D422" s="2" t="inlineStr">
@@ -9614,17 +9614,17 @@
     <row r="423">
       <c r="A423" s="3" t="inlineStr">
         <is>
-          <t>QBTS</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="B423" s="3" t="inlineStr">
         <is>
-          <t>D-Wave Quantum</t>
+          <t>PayPal</t>
         </is>
       </c>
       <c r="C423" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D423" s="3" t="inlineStr">
@@ -9636,17 +9636,17 @@
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="B424" s="2" t="inlineStr">
         <is>
-          <t>Qualcomm Inc</t>
+          <t>Qnity Electronics</t>
         </is>
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D424" s="2" t="inlineStr">
@@ -9658,17 +9658,17 @@
     <row r="425">
       <c r="A425" s="3" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>QBTS</t>
         </is>
       </c>
       <c r="B425" s="3" t="inlineStr">
         <is>
-          <t>Qualys</t>
+          <t>D-Wave Quantum</t>
         </is>
       </c>
       <c r="C425" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D425" s="3" t="inlineStr">
@@ -9680,12 +9680,12 @@
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B426" s="2" t="inlineStr">
         <is>
-          <t>QQQ ETF</t>
+          <t>Qualcomm Inc</t>
         </is>
       </c>
       <c r="C426" s="2" t="inlineStr">
@@ -9702,12 +9702,12 @@
     <row r="427">
       <c r="A427" s="3" t="inlineStr">
         <is>
-          <t>QQQM</t>
+          <t>QLYS</t>
         </is>
       </c>
       <c r="B427" s="3" t="inlineStr">
         <is>
-          <t>Invesco NASDAQ 100 ETF</t>
+          <t>Qualys</t>
         </is>
       </c>
       <c r="C427" s="3" t="inlineStr">
@@ -9724,17 +9724,17 @@
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>QTWO</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B428" s="2" t="inlineStr">
         <is>
-          <t>Q2 Holdings</t>
+          <t>QQQ ETF</t>
         </is>
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D428" s="2" t="inlineStr">
@@ -9746,13 +9746,17 @@
     <row r="429">
       <c r="A429" s="3" t="inlineStr">
         <is>
-          <t>QXO</t>
-        </is>
-      </c>
-      <c r="B429" s="3" t="n"/>
+          <t>QQQM</t>
+        </is>
+      </c>
+      <c r="B429" s="3" t="inlineStr">
+        <is>
+          <t>Invesco NASDAQ 100 ETF</t>
+        </is>
+      </c>
       <c r="C429" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D429" s="3" t="inlineStr">
@@ -9764,12 +9768,12 @@
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>RBLX</t>
+          <t>QTWO</t>
         </is>
       </c>
       <c r="B430" s="2" t="inlineStr">
         <is>
-          <t>Roblox</t>
+          <t>Q2 Holdings</t>
         </is>
       </c>
       <c r="C430" s="2" t="inlineStr">
@@ -9786,14 +9790,10 @@
     <row r="431">
       <c r="A431" s="3" t="inlineStr">
         <is>
-          <t>RBRK</t>
-        </is>
-      </c>
-      <c r="B431" s="3" t="inlineStr">
-        <is>
-          <t>Rubrik</t>
-        </is>
-      </c>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="B431" s="3" t="n"/>
       <c r="C431" s="3" t="inlineStr">
         <is>
           <t>NYSE</t>
@@ -9808,12 +9808,12 @@
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>RCL</t>
+          <t>RBLX</t>
         </is>
       </c>
       <c r="B432" s="2" t="inlineStr">
         <is>
-          <t>Royal Caribbean Cruises</t>
+          <t>Roblox</t>
         </is>
       </c>
       <c r="C432" s="2" t="inlineStr">
@@ -9830,12 +9830,12 @@
     <row r="433">
       <c r="A433" s="3" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>RBRK</t>
         </is>
       </c>
       <c r="B433" s="3" t="inlineStr">
         <is>
-          <t>Reddit</t>
+          <t>Rubrik</t>
         </is>
       </c>
       <c r="C433" s="3" t="inlineStr">
@@ -9852,12 +9852,12 @@
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>RDW</t>
+          <t>RCL</t>
         </is>
       </c>
       <c r="B434" s="2" t="inlineStr">
         <is>
-          <t>Redwire .</t>
+          <t>Royal Caribbean Cruises</t>
         </is>
       </c>
       <c r="C434" s="2" t="inlineStr">
@@ -9874,17 +9874,17 @@
     <row r="435">
       <c r="A435" s="3" t="inlineStr">
         <is>
-          <t>RGTI</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B435" s="3" t="inlineStr">
         <is>
-          <t>Rigetti Computing</t>
+          <t>Reddit</t>
         </is>
       </c>
       <c r="C435" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D435" s="3" t="inlineStr">
@@ -9896,17 +9896,17 @@
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>RGTZ</t>
+          <t>RDW</t>
         </is>
       </c>
       <c r="B436" s="2" t="inlineStr">
         <is>
-          <t>Defiance Daily Target 2X Short RGTI ETF</t>
+          <t>Redwire .</t>
         </is>
       </c>
       <c r="C436" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D436" s="2" t="inlineStr">
@@ -9918,17 +9918,17 @@
     <row r="437">
       <c r="A437" s="3" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>RGTI</t>
         </is>
       </c>
       <c r="B437" s="3" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>Rigetti Computing</t>
         </is>
       </c>
       <c r="C437" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D437" s="3" t="inlineStr">
@@ -9940,17 +9940,17 @@
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>RIO</t>
+          <t>RGTZ</t>
         </is>
       </c>
       <c r="B438" s="2" t="inlineStr">
         <is>
-          <t>Rio Tinto</t>
+          <t>Defiance Daily Target 2X Short RGTI ETF</t>
         </is>
       </c>
       <c r="C438" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D438" s="2" t="inlineStr">
@@ -9962,17 +9962,17 @@
     <row r="439">
       <c r="A439" s="3" t="inlineStr">
         <is>
-          <t>RIVN</t>
+          <t>RH</t>
         </is>
       </c>
       <c r="B439" s="3" t="inlineStr">
         <is>
-          <t>Rivian Automotive</t>
+          <t>RH</t>
         </is>
       </c>
       <c r="C439" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D439" s="3" t="inlineStr">
@@ -9984,12 +9984,12 @@
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>RJF</t>
+          <t>RIO</t>
         </is>
       </c>
       <c r="B440" s="2" t="inlineStr">
         <is>
-          <t>Raymond James Financial</t>
+          <t>Rio Tinto</t>
         </is>
       </c>
       <c r="C440" s="2" t="inlineStr">
@@ -10006,12 +10006,12 @@
     <row r="441">
       <c r="A441" s="3" t="inlineStr">
         <is>
-          <t>RKLB</t>
+          <t>RIVN</t>
         </is>
       </c>
       <c r="B441" s="3" t="inlineStr">
         <is>
-          <t>Rocket Lab</t>
+          <t>Rivian Automotive</t>
         </is>
       </c>
       <c r="C441" s="3" t="inlineStr">
@@ -10028,12 +10028,12 @@
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>RL</t>
+          <t>RJF</t>
         </is>
       </c>
       <c r="B442" s="2" t="inlineStr">
         <is>
-          <t>Ralph Lauren</t>
+          <t>Raymond James Financial</t>
         </is>
       </c>
       <c r="C442" s="2" t="inlineStr">
@@ -10050,12 +10050,12 @@
     <row r="443">
       <c r="A443" s="3" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>RKLB</t>
         </is>
       </c>
       <c r="B443" s="3" t="inlineStr">
         <is>
-          <t>Roku</t>
+          <t>Rocket Lab</t>
         </is>
       </c>
       <c r="C443" s="3" t="inlineStr">
@@ -10072,17 +10072,17 @@
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>RL</t>
         </is>
       </c>
       <c r="B444" s="2" t="inlineStr">
         <is>
-          <t>Roper Technologies</t>
+          <t>Ralph Lauren</t>
         </is>
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
@@ -10094,12 +10094,12 @@
     <row r="445">
       <c r="A445" s="3" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="B445" s="3" t="inlineStr">
         <is>
-          <t>Ross Stores</t>
+          <t>Roku</t>
         </is>
       </c>
       <c r="C445" s="3" t="inlineStr">
@@ -10116,12 +10116,12 @@
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>RPAY</t>
+          <t>ROP</t>
         </is>
       </c>
       <c r="B446" s="2" t="inlineStr">
         <is>
-          <t>Repay Holdings</t>
+          <t>Roper Technologies</t>
         </is>
       </c>
       <c r="C446" s="2" t="inlineStr">
@@ -10138,17 +10138,17 @@
     <row r="447">
       <c r="A447" s="3" t="inlineStr">
         <is>
-          <t>RRX</t>
+          <t>ROST</t>
         </is>
       </c>
       <c r="B447" s="3" t="inlineStr">
         <is>
-          <t>Regal Rexnord</t>
+          <t>Ross Stores</t>
         </is>
       </c>
       <c r="C447" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D447" s="3" t="inlineStr">
@@ -10160,17 +10160,17 @@
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>RSG</t>
+          <t>RPAY</t>
         </is>
       </c>
       <c r="B448" s="2" t="inlineStr">
         <is>
-          <t>Republic Services</t>
+          <t>Repay Holdings</t>
         </is>
       </c>
       <c r="C448" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D448" s="2" t="inlineStr">
@@ -10182,12 +10182,12 @@
     <row r="449">
       <c r="A449" s="3" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>RRX</t>
         </is>
       </c>
       <c r="B449" s="3" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>Regal Rexnord</t>
         </is>
       </c>
       <c r="C449" s="3" t="inlineStr">
@@ -10204,12 +10204,12 @@
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>RSG</t>
         </is>
       </c>
       <c r="B450" s="2" t="inlineStr">
         <is>
-          <t>SentinelOne</t>
+          <t>Republic Services</t>
         </is>
       </c>
       <c r="C450" s="2" t="inlineStr">
@@ -10226,12 +10226,12 @@
     <row r="451">
       <c r="A451" s="3" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="B451" s="3" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="C451" s="3" t="inlineStr">
@@ -10248,17 +10248,17 @@
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>SATS</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>EchoStar</t>
+          <t>SentinelOne</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D452" s="2" t="inlineStr">
@@ -10270,12 +10270,12 @@
     <row r="453">
       <c r="A453" s="3" t="inlineStr">
         <is>
-          <t>SCCO</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B453" s="3" t="inlineStr">
         <is>
-          <t>Southern Copper</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="C453" s="3" t="inlineStr">
@@ -10292,17 +10292,17 @@
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>SCHW</t>
+          <t>SATS</t>
         </is>
       </c>
       <c r="B454" s="2" t="inlineStr">
         <is>
-          <t>Charles Schwab</t>
+          <t>EchoStar</t>
         </is>
       </c>
       <c r="C454" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D454" s="2" t="inlineStr">
@@ -10314,17 +10314,17 @@
     <row r="455">
       <c r="A455" s="3" t="inlineStr">
         <is>
-          <t>SCVL</t>
+          <t>SCCO</t>
         </is>
       </c>
       <c r="B455" s="3" t="inlineStr">
         <is>
-          <t>Shoe Carnival</t>
+          <t>Southern Copper</t>
         </is>
       </c>
       <c r="C455" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D455" s="3" t="inlineStr">
@@ -10336,17 +10336,17 @@
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>SEDG</t>
+          <t>SCHW</t>
         </is>
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>SolarEdge</t>
+          <t>Charles Schwab</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
@@ -10358,12 +10358,12 @@
     <row r="457">
       <c r="A457" s="3" t="inlineStr">
         <is>
-          <t>SERV</t>
+          <t>SCVL</t>
         </is>
       </c>
       <c r="B457" s="3" t="inlineStr">
         <is>
-          <t>Serve Robotics</t>
+          <t>Shoe Carnival</t>
         </is>
       </c>
       <c r="C457" s="3" t="inlineStr">
@@ -10380,17 +10380,17 @@
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>SEDG</t>
         </is>
       </c>
       <c r="B458" s="2" t="inlineStr">
         <is>
-          <t>Stifel Financial</t>
+          <t>SolarEdge</t>
         </is>
       </c>
       <c r="C458" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D458" s="2" t="inlineStr">
@@ -10402,12 +10402,12 @@
     <row r="459">
       <c r="A459" s="3" t="inlineStr">
         <is>
-          <t>SFD</t>
+          <t>SERV</t>
         </is>
       </c>
       <c r="B459" s="3" t="inlineStr">
         <is>
-          <t>Smithfield Foods</t>
+          <t>Serve Robotics</t>
         </is>
       </c>
       <c r="C459" s="3" t="inlineStr">
@@ -10424,12 +10424,12 @@
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>SHAK</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="B460" s="2" t="inlineStr">
         <is>
-          <t>Shake Shack</t>
+          <t>Stifel Financial</t>
         </is>
       </c>
       <c r="C460" s="2" t="inlineStr">
@@ -10446,17 +10446,17 @@
     <row r="461">
       <c r="A461" s="3" t="inlineStr">
         <is>
-          <t>SHEL</t>
+          <t>SFD</t>
         </is>
       </c>
       <c r="B461" s="3" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>Smithfield Foods</t>
         </is>
       </c>
       <c r="C461" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D461" s="3" t="inlineStr">
@@ -10468,17 +10468,17 @@
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>SHAK</t>
         </is>
       </c>
       <c r="B462" s="2" t="inlineStr">
         <is>
-          <t>Shopify</t>
+          <t>Shake Shack</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D462" s="2" t="inlineStr">
@@ -10490,17 +10490,17 @@
     <row r="463">
       <c r="A463" s="3" t="inlineStr">
         <is>
-          <t>SHY</t>
+          <t>SHEL</t>
         </is>
       </c>
       <c r="B463" s="3" t="inlineStr">
         <is>
-          <t>iShares 1-3 Year Treasury Bond ETF</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="C463" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D463" s="3" t="inlineStr">
@@ -10512,17 +10512,17 @@
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>SIG</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="B464" s="2" t="inlineStr">
         <is>
-          <t>Signet Jewelers</t>
+          <t>Shopify</t>
         </is>
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
@@ -10534,12 +10534,12 @@
     <row r="465">
       <c r="A465" s="3" t="inlineStr">
         <is>
-          <t>SIMO</t>
+          <t>SHY</t>
         </is>
       </c>
       <c r="B465" s="3" t="inlineStr">
         <is>
-          <t>Silicon Motion Technology .</t>
+          <t>iShares 1-3 Year Treasury Bond ETF</t>
         </is>
       </c>
       <c r="C465" s="3" t="inlineStr">
@@ -10556,17 +10556,17 @@
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>SKYT</t>
+          <t>SIG</t>
         </is>
       </c>
       <c r="B466" s="2" t="inlineStr">
         <is>
-          <t>SkyWater Technology</t>
+          <t>Signet Jewelers</t>
         </is>
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
@@ -10578,17 +10578,17 @@
     <row r="467">
       <c r="A467" s="3" t="inlineStr">
         <is>
-          <t>SLVYY</t>
+          <t>SIMO</t>
         </is>
       </c>
       <c r="B467" s="3" t="inlineStr">
         <is>
-          <t>Solvay</t>
+          <t>Silicon Motion Technology .</t>
         </is>
       </c>
       <c r="C467" s="3" t="inlineStr">
         <is>
-          <t>OTC</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D467" s="3" t="inlineStr">
@@ -10600,12 +10600,12 @@
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>SKYT</t>
         </is>
       </c>
       <c r="B468" s="2" t="inlineStr">
         <is>
-          <t>Super Micro Computer</t>
+          <t>SkyWater Technology</t>
         </is>
       </c>
       <c r="C468" s="2" t="inlineStr">
@@ -10622,17 +10622,17 @@
     <row r="469">
       <c r="A469" s="3" t="inlineStr">
         <is>
-          <t>SMH</t>
+          <t>SLVYY</t>
         </is>
       </c>
       <c r="B469" s="3" t="inlineStr">
         <is>
-          <t>VanEck Semiconductor ETF</t>
+          <t>Solvay</t>
         </is>
       </c>
       <c r="C469" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>OTC</t>
         </is>
       </c>
       <c r="D469" s="3" t="inlineStr">
@@ -10644,12 +10644,12 @@
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>SMPL</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B470" s="2" t="inlineStr">
         <is>
-          <t>Simply Good Foods Co.</t>
+          <t>Super Micro Computer</t>
         </is>
       </c>
       <c r="C470" s="2" t="inlineStr">
@@ -10666,17 +10666,17 @@
     <row r="471">
       <c r="A471" s="3" t="inlineStr">
         <is>
-          <t>SMR</t>
+          <t>SMH</t>
         </is>
       </c>
       <c r="B471" s="3" t="inlineStr">
         <is>
-          <t>NuScale</t>
+          <t>VanEck Semiconductor ETF</t>
         </is>
       </c>
       <c r="C471" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D471" s="3" t="inlineStr">
@@ -10688,12 +10688,12 @@
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>SMX</t>
+          <t>SMPL</t>
         </is>
       </c>
       <c r="B472" s="2" t="inlineStr">
         <is>
-          <t>This message is a paid advertisement for SMX</t>
+          <t>Simply Good Foods Co.</t>
         </is>
       </c>
       <c r="C472" s="2" t="inlineStr">
@@ -10710,17 +10710,17 @@
     <row r="473">
       <c r="A473" s="3" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>SMR</t>
         </is>
       </c>
       <c r="B473" s="3" t="inlineStr">
         <is>
-          <t>SanDisk</t>
+          <t>NuScale</t>
         </is>
       </c>
       <c r="C473" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D473" s="3" t="inlineStr">
@@ -10732,17 +10732,17 @@
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>SMX</t>
         </is>
       </c>
       <c r="B474" s="2" t="inlineStr">
         <is>
-          <t>Snowflake</t>
+          <t>This message is a paid advertisement for SMX</t>
         </is>
       </c>
       <c r="C474" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D474" s="2" t="inlineStr">
@@ -10754,12 +10754,12 @@
     <row r="475">
       <c r="A475" s="3" t="inlineStr">
         <is>
-          <t>SOFI</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B475" s="3" t="inlineStr">
         <is>
-          <t>SoFi Technologies</t>
+          <t>SanDisk</t>
         </is>
       </c>
       <c r="C475" s="3" t="inlineStr">
@@ -10776,17 +10776,17 @@
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>SOLS</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B476" s="2" t="inlineStr">
         <is>
-          <t>Solstice Advanced Materials</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="C476" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D476" s="2" t="inlineStr">
@@ -10798,12 +10798,12 @@
     <row r="477">
       <c r="A477" s="3" t="inlineStr">
         <is>
-          <t>SOUN</t>
+          <t>SOFI</t>
         </is>
       </c>
       <c r="B477" s="3" t="inlineStr">
         <is>
-          <t>SoundHound AI</t>
+          <t>SoFi Technologies</t>
         </is>
       </c>
       <c r="C477" s="3" t="inlineStr">
@@ -10820,12 +10820,12 @@
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>SOLS</t>
         </is>
       </c>
       <c r="B478" s="2" t="inlineStr">
         <is>
-          <t>iShares Semiconductor ETF</t>
+          <t>Solstice Advanced Materials</t>
         </is>
       </c>
       <c r="C478" s="2" t="inlineStr">
@@ -10842,17 +10842,17 @@
     <row r="479">
       <c r="A479" s="3" t="inlineStr">
         <is>
-          <t>SPOT</t>
+          <t>SOUN</t>
         </is>
       </c>
       <c r="B479" s="3" t="inlineStr">
         <is>
-          <t>Spotify Technology</t>
+          <t>SoundHound AI</t>
         </is>
       </c>
       <c r="C479" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D479" s="3" t="inlineStr">
@@ -10864,13 +10864,17 @@
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="B480" s="2" t="n"/>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="B480" s="2" t="inlineStr">
+        <is>
+          <t>iShares Semiconductor ETF</t>
+        </is>
+      </c>
       <c r="C480" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D480" s="2" t="inlineStr">
@@ -10882,17 +10886,17 @@
     <row r="481">
       <c r="A481" s="3" t="inlineStr">
         <is>
-          <t>SQQQ</t>
+          <t>SPOT</t>
         </is>
       </c>
       <c r="B481" s="3" t="inlineStr">
         <is>
-          <t>ProShares UltraPro Short QQQ</t>
+          <t>Spotify Technology</t>
         </is>
       </c>
       <c r="C481" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D481" s="3" t="inlineStr">
@@ -10904,17 +10908,13 @@
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>SSP</t>
-        </is>
-      </c>
-      <c r="B482" s="2" t="inlineStr">
-        <is>
-          <t>E.W. Scripps</t>
-        </is>
-      </c>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="B482" s="2" t="n"/>
       <c r="C482" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D482" s="2" t="inlineStr">
@@ -10926,12 +10926,12 @@
     <row r="483">
       <c r="A483" s="3" t="inlineStr">
         <is>
-          <t>SSYS</t>
+          <t>SQQQ</t>
         </is>
       </c>
       <c r="B483" s="3" t="inlineStr">
         <is>
-          <t>Stratasys</t>
+          <t>ProShares UltraPro Short QQQ</t>
         </is>
       </c>
       <c r="C483" s="3" t="inlineStr">
@@ -10948,17 +10948,17 @@
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>STLA</t>
+          <t>SSP</t>
         </is>
       </c>
       <c r="B484" s="2" t="inlineStr">
         <is>
-          <t>Stellantis</t>
+          <t>E.W. Scripps</t>
         </is>
       </c>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D484" s="2" t="inlineStr">
@@ -10970,17 +10970,17 @@
     <row r="485">
       <c r="A485" s="3" t="inlineStr">
         <is>
-          <t>STWD</t>
+          <t>SSYS</t>
         </is>
       </c>
       <c r="B485" s="3" t="inlineStr">
         <is>
-          <t>Starwood Property Trust</t>
+          <t>Stratasys</t>
         </is>
       </c>
       <c r="C485" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D485" s="3" t="inlineStr">
@@ -10992,17 +10992,17 @@
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>STLA</t>
         </is>
       </c>
       <c r="B486" s="2" t="inlineStr">
         <is>
-          <t>Seagate Technology</t>
+          <t>Stellantis</t>
         </is>
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
@@ -11014,10 +11014,14 @@
     <row r="487">
       <c r="A487" s="3" t="inlineStr">
         <is>
-          <t>STZ</t>
-        </is>
-      </c>
-      <c r="B487" s="3" t="n"/>
+          <t>STWD</t>
+        </is>
+      </c>
+      <c r="B487" s="3" t="inlineStr">
+        <is>
+          <t>Starwood Property Trust</t>
+        </is>
+      </c>
       <c r="C487" s="3" t="inlineStr">
         <is>
           <t>NYSE</t>
@@ -11032,17 +11036,17 @@
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>SU</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B488" s="2" t="inlineStr">
         <is>
-          <t>Suncor Energy</t>
+          <t>Seagate Technology</t>
         </is>
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -11054,17 +11058,13 @@
     <row r="489">
       <c r="A489" s="3" t="inlineStr">
         <is>
-          <t>SVC</t>
-        </is>
-      </c>
-      <c r="B489" s="3" t="inlineStr">
-        <is>
-          <t>Service Property Trust</t>
-        </is>
-      </c>
+          <t>STZ</t>
+        </is>
+      </c>
+      <c r="B489" s="3" t="n"/>
       <c r="C489" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D489" s="3" t="inlineStr">
@@ -11076,10 +11076,14 @@
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="B490" s="2" t="n"/>
+          <t>SU</t>
+        </is>
+      </c>
+      <c r="B490" s="2" t="inlineStr">
+        <is>
+          <t>Suncor Energy</t>
+        </is>
+      </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
           <t>NYSE</t>
@@ -11094,17 +11098,17 @@
     <row r="491">
       <c r="A491" s="3" t="inlineStr">
         <is>
-          <t>TAIL</t>
+          <t>SVC</t>
         </is>
       </c>
       <c r="B491" s="3" t="inlineStr">
         <is>
-          <t>Cambria Tail Risk ETF</t>
+          <t>Service Property Trust</t>
         </is>
       </c>
       <c r="C491" s="3" t="inlineStr">
         <is>
-          <t>BATS</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D491" s="3" t="inlineStr">
@@ -11116,17 +11120,13 @@
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>TALK</t>
-        </is>
-      </c>
-      <c r="B492" s="2" t="inlineStr">
-        <is>
-          <t>Talkspace</t>
-        </is>
-      </c>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B492" s="2" t="n"/>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D492" s="2" t="inlineStr">
@@ -11138,17 +11138,17 @@
     <row r="493">
       <c r="A493" s="3" t="inlineStr">
         <is>
-          <t>TAP</t>
+          <t>TAIL</t>
         </is>
       </c>
       <c r="B493" s="3" t="inlineStr">
         <is>
-          <t>Molson Coors Beverage Company</t>
+          <t>Cambria Tail Risk ETF</t>
         </is>
       </c>
       <c r="C493" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>BATS</t>
         </is>
       </c>
       <c r="D493" s="3" t="inlineStr">
@@ -11160,17 +11160,17 @@
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>TCAF</t>
+          <t>TALK</t>
         </is>
       </c>
       <c r="B494" s="2" t="inlineStr">
         <is>
-          <t>T. Rowe Price Capital Appreciation Equity ETF</t>
+          <t>Talkspace</t>
         </is>
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -11182,12 +11182,12 @@
     <row r="495">
       <c r="A495" s="3" t="inlineStr">
         <is>
-          <t>TCAI</t>
+          <t>TAP</t>
         </is>
       </c>
       <c r="B495" s="3" t="inlineStr">
         <is>
-          <t>Tortoise AI Infrastructure ETF</t>
+          <t>Molson Coors Beverage Company</t>
         </is>
       </c>
       <c r="C495" s="3" t="inlineStr">
@@ -11204,17 +11204,17 @@
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>TDOC</t>
+          <t>TCAF</t>
         </is>
       </c>
       <c r="B496" s="2" t="inlineStr">
         <is>
-          <t>Teladoc Health</t>
+          <t>T. Rowe Price Capital Appreciation Equity ETF</t>
         </is>
       </c>
       <c r="C496" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D496" s="2" t="inlineStr">
@@ -11226,17 +11226,17 @@
     <row r="497">
       <c r="A497" s="3" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>TCAI</t>
         </is>
       </c>
       <c r="B497" s="3" t="inlineStr">
         <is>
-          <t>Atlassian .</t>
+          <t>Tortoise AI Infrastructure ETF</t>
         </is>
       </c>
       <c r="C497" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D497" s="3" t="inlineStr">
@@ -11248,17 +11248,17 @@
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>TDOC</t>
         </is>
       </c>
       <c r="B498" s="2" t="inlineStr">
         <is>
-          <t>Tempus AI</t>
+          <t>Teladoc Health</t>
         </is>
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -11270,12 +11270,12 @@
     <row r="499">
       <c r="A499" s="3" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="B499" s="3" t="inlineStr">
         <is>
-          <t>Tenable Holdings</t>
+          <t>Atlassian .</t>
         </is>
       </c>
       <c r="C499" s="3" t="inlineStr">
@@ -11292,12 +11292,12 @@
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="B500" s="2" t="inlineStr">
         <is>
-          <t>Teradyne</t>
+          <t>Tempus AI</t>
         </is>
       </c>
       <c r="C500" s="2" t="inlineStr">
@@ -11314,17 +11314,17 @@
     <row r="501">
       <c r="A501" s="3" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>TENB</t>
         </is>
       </c>
       <c r="B501" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Tenable Holdings</t>
         </is>
       </c>
       <c r="C501" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D501" s="3" t="inlineStr">
@@ -11336,17 +11336,17 @@
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>THC</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B502" s="2" t="inlineStr">
         <is>
-          <t>Tenet Healthcare .</t>
+          <t>Teradyne</t>
         </is>
       </c>
       <c r="C502" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D502" s="2" t="inlineStr">
@@ -11358,17 +11358,17 @@
     <row r="503">
       <c r="A503" s="3" t="inlineStr">
         <is>
-          <t>THRY</t>
+          <t>TGT</t>
         </is>
       </c>
       <c r="B503" s="3" t="inlineStr">
         <is>
-          <t>Thryv</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="C503" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D503" s="3" t="inlineStr">
@@ -11380,12 +11380,12 @@
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>THC</t>
         </is>
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>TJX Companies</t>
+          <t>Tenet Healthcare .</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -11402,12 +11402,12 @@
     <row r="505">
       <c r="A505" s="3" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>THRY</t>
         </is>
       </c>
       <c r="B505" s="3" t="inlineStr">
         <is>
-          <t>Talen Energy</t>
+          <t>Thryv</t>
         </is>
       </c>
       <c r="C505" s="3" t="inlineStr">
@@ -11424,13 +11424,17 @@
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>TMC</t>
-        </is>
-      </c>
-      <c r="B506" s="2" t="n"/>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="B506" s="2" t="inlineStr">
+        <is>
+          <t>TJX Companies</t>
+        </is>
+      </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -11442,17 +11446,17 @@
     <row r="507">
       <c r="A507" s="3" t="inlineStr">
         <is>
-          <t>TME</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B507" s="3" t="inlineStr">
         <is>
-          <t>Tencent Music Entertainment Group</t>
+          <t>Talen Energy</t>
         </is>
       </c>
       <c r="C507" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D507" s="3" t="inlineStr">
@@ -11464,17 +11468,13 @@
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>TMO</t>
-        </is>
-      </c>
-      <c r="B508" s="2" t="inlineStr">
-        <is>
-          <t>Thermo Fisher Scientific</t>
-        </is>
-      </c>
+          <t>TMC</t>
+        </is>
+      </c>
+      <c r="B508" s="2" t="n"/>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
@@ -11486,12 +11486,12 @@
     <row r="509">
       <c r="A509" s="3" t="inlineStr">
         <is>
-          <t>TOST</t>
+          <t>TME</t>
         </is>
       </c>
       <c r="B509" s="3" t="inlineStr">
         <is>
-          <t>Toast</t>
+          <t>Tencent Music Entertainment Group</t>
         </is>
       </c>
       <c r="C509" s="3" t="inlineStr">
@@ -11508,17 +11508,17 @@
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="B510" s="2" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>Thermo Fisher Scientific</t>
         </is>
       </c>
       <c r="C510" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D510" s="2" t="inlineStr">
@@ -11530,12 +11530,12 @@
     <row r="511">
       <c r="A511" s="3" t="inlineStr">
         <is>
-          <t>TPL</t>
+          <t>TOST</t>
         </is>
       </c>
       <c r="B511" s="3" t="inlineStr">
         <is>
-          <t>Texas Pacific Land Corporation</t>
+          <t>Toast</t>
         </is>
       </c>
       <c r="C511" s="3" t="inlineStr">
@@ -11552,17 +11552,17 @@
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="B512" s="2" t="inlineStr">
         <is>
-          <t>Tootsie Roll</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="C512" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D512" s="2" t="inlineStr">
@@ -11574,12 +11574,12 @@
     <row r="513">
       <c r="A513" s="3" t="inlineStr">
         <is>
-          <t>TREX</t>
+          <t>TPL</t>
         </is>
       </c>
       <c r="B513" s="3" t="inlineStr">
         <is>
-          <t>Trex Company</t>
+          <t>Texas Pacific Land Corporation</t>
         </is>
       </c>
       <c r="C513" s="3" t="inlineStr">
@@ -11596,17 +11596,17 @@
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>TRIP</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="B514" s="2" t="inlineStr">
         <is>
-          <t>TripAdvisor</t>
+          <t>Tootsie Roll</t>
         </is>
       </c>
       <c r="C514" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D514" s="2" t="inlineStr">
@@ -11618,12 +11618,12 @@
     <row r="515">
       <c r="A515" s="3" t="inlineStr">
         <is>
-          <t>TRP</t>
+          <t>TREX</t>
         </is>
       </c>
       <c r="B515" s="3" t="inlineStr">
         <is>
-          <t>TC Energy</t>
+          <t>Trex Company</t>
         </is>
       </c>
       <c r="C515" s="3" t="inlineStr">
@@ -11640,17 +11640,17 @@
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>TRV</t>
+          <t>TRIP</t>
         </is>
       </c>
       <c r="B516" s="2" t="inlineStr">
         <is>
-          <t>Travelers Companies</t>
+          <t>TripAdvisor</t>
         </is>
       </c>
       <c r="C516" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D516" s="2" t="inlineStr">
@@ -11662,17 +11662,17 @@
     <row r="517">
       <c r="A517" s="3" t="inlineStr">
         <is>
-          <t>TSCO</t>
+          <t>TRP</t>
         </is>
       </c>
       <c r="B517" s="3" t="inlineStr">
         <is>
-          <t>Tractor Supply Company</t>
+          <t>TC Energy</t>
         </is>
       </c>
       <c r="C517" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D517" s="3" t="inlineStr">
@@ -11684,17 +11684,17 @@
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>TRV</t>
         </is>
       </c>
       <c r="B518" s="2" t="inlineStr">
         <is>
-          <t>Tower Semiconductor</t>
+          <t>Travelers Companies</t>
         </is>
       </c>
       <c r="C518" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D518" s="2" t="inlineStr">
@@ -11706,12 +11706,12 @@
     <row r="519">
       <c r="A519" s="3" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>TSCO</t>
         </is>
       </c>
       <c r="B519" s="3" t="inlineStr">
         <is>
-          <t>Tesla</t>
+          <t>Tractor Supply Company</t>
         </is>
       </c>
       <c r="C519" s="3" t="inlineStr">
@@ -11728,12 +11728,12 @@
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>TSLL</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B520" s="2" t="inlineStr">
         <is>
-          <t>Direxion Daily TSLA Bull 2X Shares ETF</t>
+          <t>Tower Semiconductor</t>
         </is>
       </c>
       <c r="C520" s="2" t="inlineStr">
@@ -11750,17 +11750,17 @@
     <row r="521">
       <c r="A521" s="3" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B521" s="3" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing Company</t>
+          <t>Tesla</t>
         </is>
       </c>
       <c r="C521" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D521" s="3" t="inlineStr">
@@ -11772,12 +11772,12 @@
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>TTD</t>
+          <t>TSLL</t>
         </is>
       </c>
       <c r="B522" s="2" t="inlineStr">
         <is>
-          <t>The Trade Desk</t>
+          <t>Direxion Daily TSLA Bull 2X Shares ETF</t>
         </is>
       </c>
       <c r="C522" s="2" t="inlineStr">
@@ -11794,17 +11794,17 @@
     <row r="523">
       <c r="A523" s="3" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B523" s="3" t="inlineStr">
         <is>
-          <t>TTM Technologies</t>
+          <t>Taiwan Semiconductor Manufacturing Company</t>
         </is>
       </c>
       <c r="C523" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D523" s="3" t="inlineStr">
@@ -11816,17 +11816,17 @@
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>TU</t>
+          <t>TTD</t>
         </is>
       </c>
       <c r="B524" s="2" t="inlineStr">
         <is>
-          <t>TELUS</t>
+          <t>The Trade Desk</t>
         </is>
       </c>
       <c r="C524" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D524" s="2" t="inlineStr">
@@ -11838,17 +11838,17 @@
     <row r="525">
       <c r="A525" s="3" t="inlineStr">
         <is>
-          <t>TWLO</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B525" s="3" t="inlineStr">
         <is>
-          <t>Twilio Inc</t>
+          <t>TTM Technologies</t>
         </is>
       </c>
       <c r="C525" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D525" s="3" t="inlineStr">
@@ -11860,13 +11860,17 @@
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>TXBC</t>
-        </is>
-      </c>
-      <c r="B526" s="2" t="n"/>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B526" s="2" t="inlineStr">
+        <is>
+          <t>TELUS</t>
+        </is>
+      </c>
       <c r="C526" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D526" s="2" t="inlineStr">
@@ -11878,17 +11882,17 @@
     <row r="527">
       <c r="A527" s="3" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>TWLO</t>
         </is>
       </c>
       <c r="B527" s="3" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Twilio Inc</t>
         </is>
       </c>
       <c r="C527" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D527" s="3" t="inlineStr">
@@ -11900,17 +11904,13 @@
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="B528" s="2" t="inlineStr">
-        <is>
-          <t>Unity Software</t>
-        </is>
-      </c>
+          <t>TXBC</t>
+        </is>
+      </c>
+      <c r="B528" s="2" t="n"/>
       <c r="C528" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D528" s="2" t="inlineStr">
@@ -11922,12 +11922,12 @@
     <row r="529">
       <c r="A529" s="3" t="inlineStr">
         <is>
-          <t>UAL</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B529" s="3" t="inlineStr">
         <is>
-          <t>'s</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="C529" s="3" t="inlineStr">
@@ -11944,12 +11944,12 @@
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B530" s="2" t="inlineStr">
         <is>
-          <t>Uber Eats</t>
+          <t>Unity Software</t>
         </is>
       </c>
       <c r="C530" s="2" t="inlineStr">
@@ -11966,17 +11966,17 @@
     <row r="531">
       <c r="A531" s="3" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>UAL</t>
         </is>
       </c>
       <c r="B531" s="3" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>'s</t>
         </is>
       </c>
       <c r="C531" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D531" s="3" t="inlineStr">
@@ -11988,17 +11988,17 @@
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>UCO</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="B532" s="2" t="inlineStr">
         <is>
-          <t>ProShares Ultra Bloomberg Crude Oil</t>
+          <t>Uber Eats</t>
         </is>
       </c>
       <c r="C532" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D532" s="2" t="inlineStr">
@@ -12010,17 +12010,17 @@
     <row r="533">
       <c r="A533" s="3" t="inlineStr">
         <is>
-          <t>UDMY</t>
+          <t>UBS</t>
         </is>
       </c>
       <c r="B533" s="3" t="inlineStr">
         <is>
-          <t>Udemy</t>
+          <t>UBS</t>
         </is>
       </c>
       <c r="C533" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D533" s="3" t="inlineStr">
@@ -12032,17 +12032,17 @@
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>UFO</t>
+          <t>UCO</t>
         </is>
       </c>
       <c r="B534" s="2" t="inlineStr">
         <is>
-          <t>Procure Space ETF</t>
+          <t>ProShares Ultra Bloomberg Crude Oil</t>
         </is>
       </c>
       <c r="C534" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D534" s="2" t="inlineStr">
@@ -12054,17 +12054,17 @@
     <row r="535">
       <c r="A535" s="3" t="inlineStr">
         <is>
-          <t>UHS</t>
+          <t>UDMY</t>
         </is>
       </c>
       <c r="B535" s="3" t="inlineStr">
         <is>
-          <t>Universal Health Services</t>
+          <t>Udemy</t>
         </is>
       </c>
       <c r="C535" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D535" s="3" t="inlineStr">
@@ -12076,17 +12076,17 @@
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>UFO</t>
         </is>
       </c>
       <c r="B536" s="2" t="inlineStr">
         <is>
-          <t>Ubiquiti</t>
+          <t>Procure Space ETF</t>
         </is>
       </c>
       <c r="C536" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D536" s="2" t="inlineStr">
@@ -12098,10 +12098,14 @@
     <row r="537">
       <c r="A537" s="3" t="inlineStr">
         <is>
-          <t>UL</t>
-        </is>
-      </c>
-      <c r="B537" s="3" t="n"/>
+          <t>UHS</t>
+        </is>
+      </c>
+      <c r="B537" s="3" t="inlineStr">
+        <is>
+          <t>Universal Health Services</t>
+        </is>
+      </c>
       <c r="C537" s="3" t="inlineStr">
         <is>
           <t>NYSE</t>
@@ -12116,17 +12120,17 @@
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>ULTA</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="B538" s="2" t="inlineStr">
         <is>
-          <t>Ulta Beauty</t>
+          <t>Ubiquiti</t>
         </is>
       </c>
       <c r="C538" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D538" s="2" t="inlineStr">
@@ -12138,14 +12142,10 @@
     <row r="539">
       <c r="A539" s="3" t="inlineStr">
         <is>
-          <t>UNF</t>
-        </is>
-      </c>
-      <c r="B539" s="3" t="inlineStr">
-        <is>
-          <t>Unifirst</t>
-        </is>
-      </c>
+          <t>UL</t>
+        </is>
+      </c>
+      <c r="B539" s="3" t="n"/>
       <c r="C539" s="3" t="inlineStr">
         <is>
           <t>NYSE</t>
@@ -12160,17 +12160,17 @@
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>UNG</t>
+          <t>ULTA</t>
         </is>
       </c>
       <c r="B540" s="2" t="inlineStr">
         <is>
-          <t>United States Natural Gas Fund</t>
+          <t>Ulta Beauty</t>
         </is>
       </c>
       <c r="C540" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D540" s="2" t="inlineStr">
@@ -12182,12 +12182,12 @@
     <row r="541">
       <c r="A541" s="3" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>UNF</t>
         </is>
       </c>
       <c r="B541" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealth</t>
+          <t>Unifirst</t>
         </is>
       </c>
       <c r="C541" s="3" t="inlineStr">
@@ -12204,17 +12204,17 @@
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>UNM</t>
+          <t>UNG</t>
         </is>
       </c>
       <c r="B542" s="2" t="inlineStr">
         <is>
-          <t>Unum Group</t>
+          <t>United States Natural Gas Fund</t>
         </is>
       </c>
       <c r="C542" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D542" s="2" t="inlineStr">
@@ -12226,17 +12226,17 @@
     <row r="543">
       <c r="A543" s="3" t="inlineStr">
         <is>
-          <t>UPST</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B543" s="3" t="inlineStr">
         <is>
-          <t>Upstart Holdings</t>
+          <t>UnitedHealth</t>
         </is>
       </c>
       <c r="C543" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D543" s="3" t="inlineStr">
@@ -12248,17 +12248,17 @@
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>USAR</t>
+          <t>UNM</t>
         </is>
       </c>
       <c r="B544" s="2" t="inlineStr">
         <is>
-          <t>USA Rare Earth</t>
+          <t>Unum Group</t>
         </is>
       </c>
       <c r="C544" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D544" s="2" t="inlineStr">
@@ -12270,12 +12270,12 @@
     <row r="545">
       <c r="A545" s="3" t="inlineStr">
         <is>
-          <t>USAU</t>
+          <t>UPST</t>
         </is>
       </c>
       <c r="B545" s="3" t="inlineStr">
         <is>
-          <t>U.S. Gold .</t>
+          <t>Upstart Holdings</t>
         </is>
       </c>
       <c r="C545" s="3" t="inlineStr">
@@ -12292,17 +12292,17 @@
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>USFD</t>
+          <t>USAR</t>
         </is>
       </c>
       <c r="B546" s="2" t="inlineStr">
         <is>
-          <t>US Foods</t>
+          <t>USA Rare Earth</t>
         </is>
       </c>
       <c r="C546" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D546" s="2" t="inlineStr">
@@ -12314,17 +12314,17 @@
     <row r="547">
       <c r="A547" s="3" t="inlineStr">
         <is>
-          <t>USMV</t>
+          <t>USAU</t>
         </is>
       </c>
       <c r="B547" s="3" t="inlineStr">
         <is>
-          <t>iShares MSCI USA Min Vol Factor ETF</t>
+          <t>U.S. Gold .</t>
         </is>
       </c>
       <c r="C547" s="3" t="inlineStr">
         <is>
-          <t>BATS</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D547" s="3" t="inlineStr">
@@ -12336,17 +12336,17 @@
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>USFD</t>
         </is>
       </c>
       <c r="B548" s="2" t="inlineStr">
         <is>
-          <t>United States Oil Fund</t>
+          <t>US Foods</t>
         </is>
       </c>
       <c r="C548" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D548" s="2" t="inlineStr">
@@ -12358,17 +12358,17 @@
     <row r="549">
       <c r="A549" s="3" t="inlineStr">
         <is>
-          <t>USOY</t>
+          <t>USMV</t>
         </is>
       </c>
       <c r="B549" s="3" t="inlineStr">
         <is>
-          <t>Defiance Oil Enhanced Options Income ETF</t>
+          <t>iShares MSCI USA Min Vol Factor ETF</t>
         </is>
       </c>
       <c r="C549" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>BATS</t>
         </is>
       </c>
       <c r="D549" s="3" t="inlineStr">
@@ -12380,12 +12380,12 @@
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>UTES</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="B550" s="2" t="inlineStr">
         <is>
-          <t>Virtus Reaves Utilities ETF</t>
+          <t>United States Oil Fund</t>
         </is>
       </c>
       <c r="C550" s="2" t="inlineStr">
@@ -12402,17 +12402,17 @@
     <row r="551">
       <c r="A551" s="3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>USOY</t>
         </is>
       </c>
       <c r="B551" s="3" t="inlineStr">
         <is>
-          <t>Visa</t>
+          <t>Defiance Oil Enhanced Options Income ETF</t>
         </is>
       </c>
       <c r="C551" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D551" s="3" t="inlineStr">
@@ -12424,12 +12424,12 @@
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>VDC</t>
+          <t>UTES</t>
         </is>
       </c>
       <c r="B552" s="2" t="inlineStr">
         <is>
-          <t>Vanguard Consumer Staples ETF</t>
+          <t>Virtus Reaves Utilities ETF</t>
         </is>
       </c>
       <c r="C552" s="2" t="inlineStr">
@@ -12446,12 +12446,12 @@
     <row r="553">
       <c r="A553" s="3" t="inlineStr">
         <is>
-          <t>VET</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B553" s="3" t="inlineStr">
         <is>
-          <t>Vermilion Energy</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="C553" s="3" t="inlineStr">
@@ -12468,17 +12468,17 @@
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>VG</t>
+          <t>VDC</t>
         </is>
       </c>
       <c r="B554" s="2" t="inlineStr">
         <is>
-          <t>Venture Global</t>
+          <t>Vanguard Consumer Staples ETF</t>
         </is>
       </c>
       <c r="C554" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D554" s="2" t="inlineStr">
@@ -12490,17 +12490,17 @@
     <row r="555">
       <c r="A555" s="3" t="inlineStr">
         <is>
-          <t>VGK</t>
+          <t>VET</t>
         </is>
       </c>
       <c r="B555" s="3" t="inlineStr">
         <is>
-          <t>Vanguard FTSE Europe ETF</t>
+          <t>Vermilion Energy</t>
         </is>
       </c>
       <c r="C555" s="3" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D555" s="3" t="inlineStr">
@@ -12512,17 +12512,17 @@
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>VICR</t>
+          <t>VG</t>
         </is>
       </c>
       <c r="B556" s="2" t="inlineStr">
         <is>
-          <t>Vicor</t>
+          <t>Venture Global</t>
         </is>
       </c>
       <c r="C556" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D556" s="2" t="inlineStr">
@@ -12534,12 +12534,12 @@
     <row r="557">
       <c r="A557" s="3" t="inlineStr">
         <is>
-          <t>VIG</t>
+          <t>VGK</t>
         </is>
       </c>
       <c r="B557" s="3" t="inlineStr">
         <is>
-          <t>Dividend Appreciation ETF</t>
+          <t>Vanguard FTSE Europe ETF</t>
         </is>
       </c>
       <c r="C557" s="3" t="inlineStr">
@@ -12556,17 +12556,17 @@
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>VIK</t>
+          <t>VICR</t>
         </is>
       </c>
       <c r="B558" s="2" t="inlineStr">
         <is>
-          <t>Viking Holdings Ltd.</t>
+          <t>Vicor</t>
         </is>
       </c>
       <c r="C558" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D558" s="2" t="inlineStr">
@@ -12578,17 +12578,17 @@
     <row r="559">
       <c r="A559" s="3" t="inlineStr">
         <is>
-          <t>VKTX</t>
+          <t>VIG</t>
         </is>
       </c>
       <c r="B559" s="3" t="inlineStr">
         <is>
-          <t>Viking Therapeutics</t>
+          <t>Dividend Appreciation ETF</t>
         </is>
       </c>
       <c r="C559" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D559" s="3" t="inlineStr">
@@ -12600,12 +12600,12 @@
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>VLO</t>
+          <t>VIK</t>
         </is>
       </c>
       <c r="B560" s="2" t="inlineStr">
         <is>
-          <t>Valero Energy</t>
+          <t>Viking Holdings Ltd.</t>
         </is>
       </c>
       <c r="C560" s="2" t="inlineStr">
@@ -12622,17 +12622,17 @@
     <row r="561">
       <c r="A561" s="3" t="inlineStr">
         <is>
-          <t>VLUE</t>
+          <t>VKTX</t>
         </is>
       </c>
       <c r="B561" s="3" t="inlineStr">
         <is>
-          <t>iShares MSCI USA Value Factor ETF</t>
+          <t>Viking Therapeutics</t>
         </is>
       </c>
       <c r="C561" s="3" t="inlineStr">
         <is>
-          <t>BATS</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D561" s="3" t="inlineStr">
@@ -12644,12 +12644,12 @@
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>VMI</t>
+          <t>VLO</t>
         </is>
       </c>
       <c r="B562" s="2" t="inlineStr">
         <is>
-          <t>Valmont Industries</t>
+          <t>Valero Energy</t>
         </is>
       </c>
       <c r="C562" s="2" t="inlineStr">
@@ -12666,17 +12666,17 @@
     <row r="563">
       <c r="A563" s="3" t="inlineStr">
         <is>
-          <t>VNOM</t>
+          <t>VLUE</t>
         </is>
       </c>
       <c r="B563" s="3" t="inlineStr">
         <is>
-          <t>Viper Energy Partners LP</t>
+          <t>iShares MSCI USA Value Factor ETF</t>
         </is>
       </c>
       <c r="C563" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>BATS</t>
         </is>
       </c>
       <c r="D563" s="3" t="inlineStr">
@@ -12688,17 +12688,17 @@
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>VNQI</t>
+          <t>VMI</t>
         </is>
       </c>
       <c r="B564" s="2" t="inlineStr">
         <is>
-          <t>Vanguard Global ex-U.S. Real Estate ETF</t>
+          <t>Valmont Industries</t>
         </is>
       </c>
       <c r="C564" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D564" s="2" t="inlineStr">
@@ -12710,12 +12710,12 @@
     <row r="565">
       <c r="A565" s="3" t="inlineStr">
         <is>
-          <t>VOD</t>
+          <t>VNOM</t>
         </is>
       </c>
       <c r="B565" s="3" t="inlineStr">
         <is>
-          <t>Vodafone</t>
+          <t>Viper Energy Partners LP</t>
         </is>
       </c>
       <c r="C565" s="3" t="inlineStr">
@@ -12732,17 +12732,17 @@
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>VOO</t>
+          <t>VNQI</t>
         </is>
       </c>
       <c r="B566" s="2" t="inlineStr">
         <is>
-          <t>P 500 ETF</t>
+          <t>Vanguard Global ex-U.S. Real Estate ETF</t>
         </is>
       </c>
       <c r="C566" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D566" s="2" t="inlineStr">
@@ -12754,17 +12754,17 @@
     <row r="567">
       <c r="A567" s="3" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>VOD</t>
         </is>
       </c>
       <c r="B567" s="3" t="inlineStr">
         <is>
-          <t>Vertiv Holdings</t>
+          <t>Vodafone</t>
         </is>
       </c>
       <c r="C567" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D567" s="3" t="inlineStr">
@@ -12776,17 +12776,17 @@
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>VSAT</t>
+          <t>VOO</t>
         </is>
       </c>
       <c r="B568" s="2" t="inlineStr">
         <is>
-          <t>Viasat</t>
+          <t>P 500 ETF</t>
         </is>
       </c>
       <c r="C568" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D568" s="2" t="inlineStr">
@@ -12798,12 +12798,12 @@
     <row r="569">
       <c r="A569" s="3" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B569" s="3" t="inlineStr">
         <is>
-          <t>Vistra</t>
+          <t>Vertiv Holdings</t>
         </is>
       </c>
       <c r="C569" s="3" t="inlineStr">
@@ -12820,10 +12820,14 @@
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>VWAV</t>
-        </is>
-      </c>
-      <c r="B570" s="2" t="n"/>
+          <t>VSAT</t>
+        </is>
+      </c>
+      <c r="B570" s="2" t="inlineStr">
+        <is>
+          <t>Viasat</t>
+        </is>
+      </c>
       <c r="C570" s="2" t="inlineStr">
         <is>
           <t>NASDAQ</t>
@@ -12838,10 +12842,14 @@
     <row r="571">
       <c r="A571" s="3" t="inlineStr">
         <is>
-          <t>VZ</t>
-        </is>
-      </c>
-      <c r="B571" s="3" t="n"/>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B571" s="3" t="inlineStr">
+        <is>
+          <t>Vistra</t>
+        </is>
+      </c>
       <c r="C571" s="3" t="inlineStr">
         <is>
           <t>NYSE</t>
@@ -12856,17 +12864,13 @@
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="B572" s="2" t="inlineStr">
-        <is>
-          <t>Wayfair</t>
-        </is>
-      </c>
+          <t>VWAV</t>
+        </is>
+      </c>
+      <c r="B572" s="2" t="n"/>
       <c r="C572" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D572" s="2" t="inlineStr">
@@ -12878,17 +12882,13 @@
     <row r="573">
       <c r="A573" s="3" t="inlineStr">
         <is>
-          <t>WBD</t>
-        </is>
-      </c>
-      <c r="B573" s="3" t="inlineStr">
-        <is>
-          <t>Warner Bros. Discovery</t>
-        </is>
-      </c>
+          <t>VZ</t>
+        </is>
+      </c>
+      <c r="B573" s="3" t="n"/>
       <c r="C573" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D573" s="3" t="inlineStr">
@@ -12900,17 +12900,17 @@
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>WCBR</t>
+          <t>W</t>
         </is>
       </c>
       <c r="B574" s="2" t="inlineStr">
         <is>
-          <t>WisdomTree Cybersecurity Fund</t>
+          <t>Wayfair</t>
         </is>
       </c>
       <c r="C574" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D574" s="2" t="inlineStr">
@@ -12922,12 +12922,12 @@
     <row r="575">
       <c r="A575" s="3" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>WBD</t>
         </is>
       </c>
       <c r="B575" s="3" t="inlineStr">
         <is>
-          <t>Workday</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="C575" s="3" t="inlineStr">
@@ -12944,12 +12944,12 @@
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>WCBR</t>
         </is>
       </c>
       <c r="B576" s="2" t="inlineStr">
         <is>
-          <t>Western Digital</t>
+          <t>WisdomTree Cybersecurity Fund</t>
         </is>
       </c>
       <c r="C576" s="2" t="inlineStr">
@@ -12966,12 +12966,12 @@
     <row r="577">
       <c r="A577" s="3" t="inlineStr">
         <is>
-          <t>WDFC</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B577" s="3" t="inlineStr">
         <is>
-          <t>WD-40 Company</t>
+          <t>Workday</t>
         </is>
       </c>
       <c r="C577" s="3" t="inlineStr">
@@ -12988,17 +12988,17 @@
     <row r="578">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>WEBS</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B578" s="2" t="inlineStr">
         <is>
-          <t>Direxion Daily Dow Jones Internet Bear 3X Shares</t>
+          <t>Western Digital</t>
         </is>
       </c>
       <c r="C578" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D578" s="2" t="inlineStr">
@@ -13010,17 +13010,17 @@
     <row r="579">
       <c r="A579" s="3" t="inlineStr">
         <is>
-          <t>WEC</t>
+          <t>WDFC</t>
         </is>
       </c>
       <c r="B579" s="3" t="inlineStr">
         <is>
-          <t>WEC Energy Group</t>
+          <t>WD-40 Company</t>
         </is>
       </c>
       <c r="C579" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D579" s="3" t="inlineStr">
@@ -13032,17 +13032,17 @@
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>WEN</t>
+          <t>WEBS</t>
         </is>
       </c>
       <c r="B580" s="2" t="inlineStr">
         <is>
-          <t>s Co.</t>
+          <t>Direxion Daily Dow Jones Internet Bear 3X Shares</t>
         </is>
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
@@ -13054,12 +13054,12 @@
     <row r="581">
       <c r="A581" s="3" t="inlineStr">
         <is>
-          <t>WFC</t>
+          <t>WEC</t>
         </is>
       </c>
       <c r="B581" s="3" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>WEC Energy Group</t>
         </is>
       </c>
       <c r="C581" s="3" t="inlineStr">
@@ -13076,17 +13076,17 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>WGO</t>
+          <t>WEN</t>
         </is>
       </c>
       <c r="B582" s="2" t="inlineStr">
         <is>
-          <t>Winnebago Industries</t>
+          <t>s Co.</t>
         </is>
       </c>
       <c r="C582" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D582" s="2" t="inlineStr">
@@ -13098,12 +13098,12 @@
     <row r="583">
       <c r="A583" s="3" t="inlineStr">
         <is>
-          <t>WHR</t>
+          <t>WFC</t>
         </is>
       </c>
       <c r="B583" s="3" t="inlineStr">
         <is>
-          <t>Whirlpool</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="C583" s="3" t="inlineStr">
@@ -13120,17 +13120,17 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>WING</t>
+          <t>WGO</t>
         </is>
       </c>
       <c r="B584" s="2" t="inlineStr">
         <is>
-          <t>Wingstop</t>
+          <t>Winnebago Industries</t>
         </is>
       </c>
       <c r="C584" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D584" s="2" t="inlineStr">
@@ -13142,12 +13142,12 @@
     <row r="585">
       <c r="A585" s="3" t="inlineStr">
         <is>
-          <t>WM</t>
+          <t>WHR</t>
         </is>
       </c>
       <c r="B585" s="3" t="inlineStr">
         <is>
-          <t>Waste Management</t>
+          <t>Whirlpool</t>
         </is>
       </c>
       <c r="C585" s="3" t="inlineStr">
@@ -13164,12 +13164,12 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>WING</t>
         </is>
       </c>
       <c r="B586" s="2" t="inlineStr">
         <is>
-          <t>Walmart</t>
+          <t>Wingstop</t>
         </is>
       </c>
       <c r="C586" s="2" t="inlineStr">
@@ -13186,12 +13186,12 @@
     <row r="587">
       <c r="A587" s="3" t="inlineStr">
         <is>
-          <t>WRB</t>
+          <t>WM</t>
         </is>
       </c>
       <c r="B587" s="3" t="inlineStr">
         <is>
-          <t>W.R. Berkley</t>
+          <t>Waste Management</t>
         </is>
       </c>
       <c r="C587" s="3" t="inlineStr">
@@ -13208,12 +13208,12 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>WWD</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B588" s="2" t="inlineStr">
         <is>
-          <t>Woodward</t>
+          <t>Walmart</t>
         </is>
       </c>
       <c r="C588" s="2" t="inlineStr">
@@ -13230,17 +13230,17 @@
     <row r="589">
       <c r="A589" s="3" t="inlineStr">
         <is>
-          <t>WYNN</t>
+          <t>WRB</t>
         </is>
       </c>
       <c r="B589" s="3" t="inlineStr">
         <is>
-          <t>Wynn Resorts Ltd.</t>
+          <t>W.R. Berkley</t>
         </is>
       </c>
       <c r="C589" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D589" s="3" t="inlineStr">
@@ -13252,17 +13252,17 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>XAR</t>
+          <t>WWD</t>
         </is>
       </c>
       <c r="B590" s="2" t="inlineStr">
         <is>
-          <t>Defense ETF</t>
+          <t>Woodward</t>
         </is>
       </c>
       <c r="C590" s="2" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D590" s="2" t="inlineStr">
@@ -13274,12 +13274,12 @@
     <row r="591">
       <c r="A591" s="3" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>WYNN</t>
         </is>
       </c>
       <c r="B591" s="3" t="inlineStr">
         <is>
-          <t>Xcel Energy</t>
+          <t>Wynn Resorts Ltd.</t>
         </is>
       </c>
       <c r="C591" s="3" t="inlineStr">
@@ -13296,10 +13296,14 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>XLE</t>
-        </is>
-      </c>
-      <c r="B592" s="2" t="n"/>
+          <t>XAR</t>
+        </is>
+      </c>
+      <c r="B592" s="2" t="inlineStr">
+        <is>
+          <t>Defense ETF</t>
+        </is>
+      </c>
       <c r="C592" s="2" t="inlineStr">
         <is>
           <t>NYSEARCA</t>
@@ -13314,17 +13318,17 @@
     <row r="593">
       <c r="A593" s="3" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B593" s="3" t="inlineStr">
         <is>
-          <t>Financial Select Sector SPDR Fund</t>
+          <t>Xcel Energy</t>
         </is>
       </c>
       <c r="C593" s="3" t="inlineStr">
         <is>
-          <t>NYSEARCA</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D593" s="3" t="inlineStr">
@@ -13336,14 +13340,10 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>XLK</t>
-        </is>
-      </c>
-      <c r="B594" s="2" t="inlineStr">
-        <is>
-          <t>State Street Technology Sector SPDR ETF</t>
-        </is>
-      </c>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="B594" s="2" t="n"/>
       <c r="C594" s="2" t="inlineStr">
         <is>
           <t>NYSEARCA</t>
@@ -13358,12 +13358,12 @@
     <row r="595">
       <c r="A595" s="3" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="B595" s="3" t="inlineStr">
         <is>
-          <t>Utilities Select Sector SPDR Fund</t>
+          <t>Financial Select Sector SPDR Fund</t>
         </is>
       </c>
       <c r="C595" s="3" t="inlineStr">
@@ -13380,12 +13380,12 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B596" s="2" t="inlineStr">
         <is>
-          <t>Health Care Select SPDR Fund ETF</t>
+          <t>State Street Technology Sector SPDR ETF</t>
         </is>
       </c>
       <c r="C596" s="2" t="inlineStr">
@@ -13402,12 +13402,12 @@
     <row r="597">
       <c r="A597" s="3" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="B597" s="3" t="inlineStr">
         <is>
-          <t>Consumer Discretionary Select Sector SPDR Fund</t>
+          <t>Utilities Select Sector SPDR Fund</t>
         </is>
       </c>
       <c r="C597" s="3" t="inlineStr">
@@ -13424,17 +13424,17 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="B598" s="2" t="inlineStr">
         <is>
-          <t>ExxonMobil</t>
+          <t>Health Care Select SPDR Fund ETF</t>
         </is>
       </c>
       <c r="C598" s="2" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D598" s="2" t="inlineStr">
@@ -13446,12 +13446,12 @@
     <row r="599">
       <c r="A599" s="3" t="inlineStr">
         <is>
-          <t>XRT</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="B599" s="3" t="inlineStr">
         <is>
-          <t>SPDR S&amp;P Retail ETF</t>
+          <t>Consumer Discretionary Select Sector SPDR Fund</t>
         </is>
       </c>
       <c r="C599" s="3" t="inlineStr">
@@ -13468,12 +13468,12 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>XXI</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B600" s="2" t="inlineStr">
         <is>
-          <t>Twenty One Capital</t>
+          <t>ExxonMobil</t>
         </is>
       </c>
       <c r="C600" s="2" t="inlineStr">
@@ -13490,17 +13490,17 @@
     <row r="601">
       <c r="A601" s="3" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>XRT</t>
         </is>
       </c>
       <c r="B601" s="3" t="inlineStr">
         <is>
-          <t>Block</t>
+          <t>SPDR S&amp;P Retail ETF</t>
         </is>
       </c>
       <c r="C601" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NYSEARCA</t>
         </is>
       </c>
       <c r="D601" s="3" t="inlineStr">
@@ -13512,12 +13512,12 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>YPF</t>
+          <t>XXI</t>
         </is>
       </c>
       <c r="B602" s="2" t="inlineStr">
         <is>
-          <t>nima</t>
+          <t>Twenty One Capital</t>
         </is>
       </c>
       <c r="C602" s="2" t="inlineStr">
@@ -13534,17 +13534,17 @@
     <row r="603">
       <c r="A603" s="3" t="inlineStr">
         <is>
-          <t>ZD</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="B603" s="3" t="inlineStr">
         <is>
-          <t>Ziff Davis</t>
+          <t>Block</t>
         </is>
       </c>
       <c r="C603" s="3" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D603" s="3" t="inlineStr">
@@ -13556,17 +13556,17 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>ZENA</t>
+          <t>YPF</t>
         </is>
       </c>
       <c r="B604" s="2" t="inlineStr">
         <is>
-          <t>And Small-Cap Defense Company ZenaTech</t>
+          <t>nima</t>
         </is>
       </c>
       <c r="C604" s="2" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="D604" s="2" t="inlineStr">
@@ -13578,17 +13578,17 @@
     <row r="605">
       <c r="A605" s="3" t="inlineStr">
         <is>
-          <t>ZETA</t>
+          <t>ZD</t>
         </is>
       </c>
       <c r="B605" s="3" t="inlineStr">
         <is>
-          <t>Zeta Global</t>
+          <t>Ziff Davis</t>
         </is>
       </c>
       <c r="C605" s="3" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D605" s="3" t="inlineStr">
@@ -13600,12 +13600,12 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>ZG</t>
+          <t>ZENA</t>
         </is>
       </c>
       <c r="B606" s="2" t="inlineStr">
         <is>
-          <t>Zillow Group</t>
+          <t>And Small-Cap Defense Company ZenaTech</t>
         </is>
       </c>
       <c r="C606" s="2" t="inlineStr">
@@ -13622,12 +13622,12 @@
     <row r="607">
       <c r="A607" s="3" t="inlineStr">
         <is>
-          <t>ZIM</t>
+          <t>ZETA</t>
         </is>
       </c>
       <c r="B607" s="3" t="inlineStr">
         <is>
-          <t>ZIM Integrated Shipping Services Ltd.</t>
+          <t>Zeta Global</t>
         </is>
       </c>
       <c r="C607" s="3" t="inlineStr">
@@ -13644,20 +13644,64 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
+          <t>ZG</t>
+        </is>
+      </c>
+      <c r="B608" s="2" t="inlineStr">
+        <is>
+          <t>Zillow Group</t>
+        </is>
+      </c>
+      <c r="C608" s="2" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D608" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="3" t="inlineStr">
+        <is>
+          <t>ZIM</t>
+        </is>
+      </c>
+      <c r="B609" s="3" t="inlineStr">
+        <is>
+          <t>ZIM Integrated Shipping Services Ltd.</t>
+        </is>
+      </c>
+      <c r="C609" s="3" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="D609" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="2" t="inlineStr">
+        <is>
           <t>ZS</t>
         </is>
       </c>
-      <c r="B608" s="2" t="inlineStr">
+      <c r="B610" s="2" t="inlineStr">
         <is>
           <t>Zscaler</t>
         </is>
       </c>
-      <c r="C608" s="2" t="inlineStr">
-        <is>
-          <t>NASDAQ</t>
-        </is>
-      </c>
-      <c r="D608" s="2" t="inlineStr">
+      <c r="C610" s="2" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D610" s="2" t="inlineStr">
         <is>
           <t>2026-06-06</t>
         </is>
@@ -13830,7 +13874,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16">
@@ -13960,7 +14004,7 @@
         </is>
       </c>
       <c r="B28" s="1" t="n">
-        <v>607</v>
+        <v>609</v>
       </c>
     </row>
   </sheetData>

</xml_diff>